<commit_message>
Add monthly expense list and actual license costs to finance plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Akadz6dHFFBjLyvCaxEhap
</commit_message>
<xml_diff>
--- a/out/Finance_and_Accountability_Plan.xlsx
+++ b/out/Finance_and_Accountability_Plan.xlsx
@@ -82,11 +82,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Fill in what you spend per week on rent, food, gas, etc. Left at $0 the plan is overly optimistic.</t>
+          <t xml:space="preserve">Monthly total × 12 ÷ 52 = weekly.</t>
         </r>
       </text>
     </comment>
-    <comment ref="B10" authorId="0">
+    <comment ref="B12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -94,11 +94,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Fill in subscription / reset / activation costs, spread per week.</t>
+          <t xml:space="preserve">(Amount needed + license costs) ÷ 12 weeks. This is what you must keep after expenses each week.</t>
         </r>
       </text>
     </comment>
-    <comment ref="B14" authorId="0">
+    <comment ref="B19" authorId="0">
       <text>
         <r>
           <rPr>
@@ -106,11 +106,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">The CE Shop Oregon pre-license course (estimate — use your real price)</t>
+          <t xml:space="preserve">Pre-license package — $300, from you</t>
         </r>
       </text>
     </comment>
-    <comment ref="B21" authorId="0">
+    <comment ref="B26" authorId="0">
       <text>
         <r>
           <rPr>
@@ -118,11 +118,11 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">PSI exam fee (estimate — confirm with PSI)</t>
+          <t xml:space="preserve">PSI exam fee — ESTIMATE, confirm with PSI and replace</t>
         </r>
       </text>
     </comment>
-    <comment ref="B23" authorId="0">
+    <comment ref="B29" authorId="0">
       <text>
         <r>
           <rPr>
@@ -130,7 +130,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">License application + fingerprints (estimate — confirm at oregon.gov/rea)</t>
+          <t xml:space="preserve">License application fee — $300, from you (fingerprinting may be extra)</t>
         </r>
       </text>
     </comment>
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="73">
   <si>
     <t xml:space="preserve">Savings Plan — $2,600 → $6,000+ by Jan 1, 2027</t>
   </si>
@@ -184,45 +184,69 @@
     <t xml:space="preserve">Assumptions</t>
   </si>
   <si>
+    <t xml:space="preserve">Monthly expenses (fill in)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Starting balance</t>
   </si>
   <si>
-    <t xml:space="preserve">From you (Oct 12, 2026).</t>
+    <t xml:space="preserve">Rent / housing</t>
   </si>
   <si>
     <t xml:space="preserve">Savings goal</t>
   </si>
   <si>
-    <t xml:space="preserve">From you: $6,000+ (need +$3,400).</t>
+    <t xml:space="preserve">Utilities</t>
   </si>
   <si>
     <t xml:space="preserve">Trading income / week — low case</t>
   </si>
   <si>
-    <t xml:space="preserve">From you: Topstep $1–2k/week. Not guaranteed; payouts follow Topstep's rules and schedule.</t>
+    <t xml:space="preserve">Phone</t>
   </si>
   <si>
     <t xml:space="preserve">Trading income / week — high case</t>
   </si>
   <si>
-    <t xml:space="preserve">From you: Topstep $1–2k/week.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Living spending / week (fill in)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fill in what you spend per week on rent, food, gas, etc. Left at $0 the plan is overly optimistic.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Topstep fees / week (fill in)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fill in subscription / reset / activation costs, spread per week.</t>
+    <t xml:space="preserve">Car payment + insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expenses / week (from monthly list →)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topstep fees: include in the monthly list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Groceries / food</t>
   </si>
   <si>
     <t xml:space="preserve">Amount still needed</t>
   </si>
   <si>
+    <t xml:space="preserve">Gym membership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly savings needed to hit goal by Jan 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subscriptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly trading income needed (incl. expenses)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Topstep subscription / resets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other / fun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total per month</t>
+  </si>
+  <si>
     <t xml:space="preserve">Week of</t>
   </si>
   <si>
@@ -241,7 +265,7 @@
     <t xml:space="preserve">Other income</t>
   </si>
   <si>
-    <t xml:space="preserve">Actual spending</t>
+    <t xml:space="preserve">Actual expenses</t>
   </si>
   <si>
     <t xml:space="preserve">Actual license + trading costs</t>
@@ -283,10 +307,13 @@
     <t xml:space="preserve">Notes:</t>
   </si>
   <si>
+    <t xml:space="preserve">• Fill in the Monthly expenses list — weekly expenses come from it and every plan balance subtracts them.</t>
+  </si>
+  <si>
     <t xml:space="preserve">• Trading income is not guaranteed. Size your plan so the goal still works if a week is $0 — the low case is your real plan, the high case is a bonus.</t>
   </si>
   <si>
-    <t xml:space="preserve">• License costs are estimates; replace them with your real prices once you buy the course / book the exam.</t>
+    <t xml:space="preserve">• License costs: $300 package and $300 application are from you; the $150 exam fee is an estimate — replace it with the real price.</t>
   </si>
   <si>
     <t xml:space="preserve">• Blue = inputs, black = formulas. Enter weekly totals in the yellow Actual columns.</t>
@@ -379,7 +406,7 @@
     <numFmt numFmtId="168" formatCode="0"/>
     <numFmt numFmtId="169" formatCode="General"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -440,6 +467,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="8"/>
       <color rgb="FF808080"/>
@@ -450,6 +484,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
+      <color rgb="FFC00000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -582,7 +617,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -607,23 +642,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -631,31 +674,23 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -663,19 +698,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -687,7 +726,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -695,7 +734,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -760,7 +799,7 @@
     <indexedColors>
       <rgbColor rgb="FF000000"/>
       <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FFC00000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -999,7 +1038,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1028,591 +1067,668 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="D4" s="3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>2600</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>4</v>
+      <c r="D5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>6000</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>6</v>
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>1000</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>8</v>
+      <c r="D7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>2000</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>10</v>
+      <c r="D8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="6" t="s">
         <v>12</v>
       </c>
+      <c r="B9" s="6" t="n">
+        <f aca="false">E15*12/52</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>14</v>
       </c>
+      <c r="D10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="8" t="n">
+      <c r="A11" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="9" t="n">
         <f aca="false">$B$6-$B$5</f>
         <v>3400</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="9" t="s">
+      <c r="D11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="E11" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="B12" s="9" t="n">
+        <f aca="false">(B11+SUM(B19:B30))/12</f>
+        <v>345.833333333333</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="B13" s="10" t="n">
+        <f aca="false">B12+B9</f>
+        <v>345.833333333333</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="E13" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="E14" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D15" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I13" s="9" t="s">
+      <c r="E15" s="6" t="n">
+        <f aca="false">SUM(E5:E14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="B18" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="C18" s="11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
+      <c r="D18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="K18" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="n">
         <v>46307</v>
       </c>
-      <c r="B14" s="11" t="n">
-        <v>400</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A14)*($B$7-$B$9-$B$10)-SUM(B$14:B14)</f>
-        <v>3200</v>
-      </c>
-      <c r="D14" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A14)*($B$8-$B$9-$B$10)-SUM(B$14:B14)</f>
-        <v>4200</v>
-      </c>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="12" t="str">
-        <f aca="false">IF(E14="","",$B$5+SUM(E$14:F14)-SUM(G$14:H14))</f>
-        <v/>
-      </c>
-      <c r="J14" s="13" t="str">
-        <f aca="false">IF(I14="","",I14/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K14" s="14" t="str">
-        <f aca="false">IF(I14="","",IF(I14&gt;=$B$6,"GOAL HIT",IF(I14&gt;=C14,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
+      <c r="B19" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="C19" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A19)*($B$7-$B$9)-SUM(B$19:B19)</f>
+        <v>3300</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A19)*($B$8-$B$9)-SUM(B$19:B19)</f>
+        <v>4300</v>
+      </c>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="14" t="str">
+        <f aca="false">IF(E19="","",$B$5+SUM(E$19:F19)-SUM(G$19:H19))</f>
+        <v/>
+      </c>
+      <c r="J19" s="15" t="str">
+        <f aca="false">IF(I19="","",I19/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K19" s="16" t="str">
+        <f aca="false">IF(I19="","",IF(I19&gt;=$B$6,"GOAL HIT",IF(I19&gt;=C19,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="n">
         <v>46314</v>
       </c>
-      <c r="B15" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A15)*($B$7-$B$9-$B$10)-SUM(B$14:B15)</f>
-        <v>4200</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A15)*($B$8-$B$9-$B$10)-SUM(B$14:B15)</f>
-        <v>6200</v>
-      </c>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="12" t="str">
-        <f aca="false">IF(E15="","",$B$5+SUM(E$14:F15)-SUM(G$14:H15))</f>
-        <v/>
-      </c>
-      <c r="J15" s="13" t="str">
-        <f aca="false">IF(I15="","",I15/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K15" s="14" t="str">
-        <f aca="false">IF(I15="","",IF(I15&gt;=$B$6,"GOAL HIT",IF(I15&gt;=C15,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+      <c r="B20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A20)*($B$7-$B$9)-SUM(B$19:B20)</f>
+        <v>4300</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A20)*($B$8-$B$9)-SUM(B$19:B20)</f>
+        <v>6300</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="14" t="str">
+        <f aca="false">IF(E20="","",$B$5+SUM(E$19:F20)-SUM(G$19:H20))</f>
+        <v/>
+      </c>
+      <c r="J20" s="15" t="str">
+        <f aca="false">IF(I20="","",I20/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K20" s="16" t="str">
+        <f aca="false">IF(I20="","",IF(I20&gt;=$B$6,"GOAL HIT",IF(I20&gt;=C20,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="n">
         <v>46321</v>
       </c>
-      <c r="B16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A16)*($B$7-$B$9-$B$10)-SUM(B$14:B16)</f>
-        <v>5200</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A16)*($B$8-$B$9-$B$10)-SUM(B$14:B16)</f>
-        <v>8200</v>
-      </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="12" t="str">
-        <f aca="false">IF(E16="","",$B$5+SUM(E$14:F16)-SUM(G$14:H16))</f>
-        <v/>
-      </c>
-      <c r="J16" s="13" t="str">
-        <f aca="false">IF(I16="","",I16/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K16" s="14" t="str">
-        <f aca="false">IF(I16="","",IF(I16&gt;=$B$6,"GOAL HIT",IF(I16&gt;=C16,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
+      <c r="B21" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A21)*($B$7-$B$9)-SUM(B$19:B21)</f>
+        <v>5300</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A21)*($B$8-$B$9)-SUM(B$19:B21)</f>
+        <v>8300</v>
+      </c>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="14" t="str">
+        <f aca="false">IF(E21="","",$B$5+SUM(E$19:F21)-SUM(G$19:H21))</f>
+        <v/>
+      </c>
+      <c r="J21" s="15" t="str">
+        <f aca="false">IF(I21="","",I21/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K21" s="16" t="str">
+        <f aca="false">IF(I21="","",IF(I21&gt;=$B$6,"GOAL HIT",IF(I21&gt;=C21,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="n">
         <v>46328</v>
       </c>
-      <c r="B17" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A17)*($B$7-$B$9-$B$10)-SUM(B$14:B17)</f>
-        <v>6200</v>
-      </c>
-      <c r="D17" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A17)*($B$8-$B$9-$B$10)-SUM(B$14:B17)</f>
-        <v>10200</v>
-      </c>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="12" t="str">
-        <f aca="false">IF(E17="","",$B$5+SUM(E$14:F17)-SUM(G$14:H17))</f>
-        <v/>
-      </c>
-      <c r="J17" s="13" t="str">
-        <f aca="false">IF(I17="","",I17/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K17" s="14" t="str">
-        <f aca="false">IF(I17="","",IF(I17&gt;=$B$6,"GOAL HIT",IF(I17&gt;=C17,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
+      <c r="B22" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A22)*($B$7-$B$9)-SUM(B$19:B22)</f>
+        <v>6300</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A22)*($B$8-$B$9)-SUM(B$19:B22)</f>
+        <v>10300</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="14" t="str">
+        <f aca="false">IF(E22="","",$B$5+SUM(E$19:F22)-SUM(G$19:H22))</f>
+        <v/>
+      </c>
+      <c r="J22" s="15" t="str">
+        <f aca="false">IF(I22="","",I22/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K22" s="16" t="str">
+        <f aca="false">IF(I22="","",IF(I22&gt;=$B$6,"GOAL HIT",IF(I22&gt;=C22,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="n">
         <v>46335</v>
       </c>
-      <c r="B18" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C18" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A18)*($B$7-$B$9-$B$10)-SUM(B$14:B18)</f>
-        <v>7200</v>
-      </c>
-      <c r="D18" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A18)*($B$8-$B$9-$B$10)-SUM(B$14:B18)</f>
-        <v>12200</v>
-      </c>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="12" t="str">
-        <f aca="false">IF(E18="","",$B$5+SUM(E$14:F18)-SUM(G$14:H18))</f>
-        <v/>
-      </c>
-      <c r="J18" s="13" t="str">
-        <f aca="false">IF(I18="","",I18/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K18" s="14" t="str">
-        <f aca="false">IF(I18="","",IF(I18&gt;=$B$6,"GOAL HIT",IF(I18&gt;=C18,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="n">
+      <c r="B23" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A23)*($B$7-$B$9)-SUM(B$19:B23)</f>
+        <v>7300</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A23)*($B$8-$B$9)-SUM(B$19:B23)</f>
+        <v>12300</v>
+      </c>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="14" t="str">
+        <f aca="false">IF(E23="","",$B$5+SUM(E$19:F23)-SUM(G$19:H23))</f>
+        <v/>
+      </c>
+      <c r="J23" s="15" t="str">
+        <f aca="false">IF(I23="","",I23/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K23" s="16" t="str">
+        <f aca="false">IF(I23="","",IF(I23&gt;=$B$6,"GOAL HIT",IF(I23&gt;=C23,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="n">
         <v>46342</v>
       </c>
-      <c r="B19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A19)*($B$7-$B$9-$B$10)-SUM(B$14:B19)</f>
-        <v>8200</v>
-      </c>
-      <c r="D19" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A19)*($B$8-$B$9-$B$10)-SUM(B$14:B19)</f>
-        <v>14200</v>
-      </c>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="12" t="str">
-        <f aca="false">IF(E19="","",$B$5+SUM(E$14:F19)-SUM(G$14:H19))</f>
-        <v/>
-      </c>
-      <c r="J19" s="13" t="str">
-        <f aca="false">IF(I19="","",I19/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K19" s="14" t="str">
-        <f aca="false">IF(I19="","",IF(I19&gt;=$B$6,"GOAL HIT",IF(I19&gt;=C19,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="B24" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A24)*($B$7-$B$9)-SUM(B$19:B24)</f>
+        <v>8300</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A24)*($B$8-$B$9)-SUM(B$19:B24)</f>
+        <v>14300</v>
+      </c>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="14" t="str">
+        <f aca="false">IF(E24="","",$B$5+SUM(E$19:F24)-SUM(G$19:H24))</f>
+        <v/>
+      </c>
+      <c r="J24" s="15" t="str">
+        <f aca="false">IF(I24="","",I24/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K24" s="16" t="str">
+        <f aca="false">IF(I24="","",IF(I24&gt;=$B$6,"GOAL HIT",IF(I24&gt;=C24,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="n">
         <v>46349</v>
       </c>
-      <c r="B20" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A20)*($B$7-$B$9-$B$10)-SUM(B$14:B20)</f>
-        <v>9200</v>
-      </c>
-      <c r="D20" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A20)*($B$8-$B$9-$B$10)-SUM(B$14:B20)</f>
-        <v>16200</v>
-      </c>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="12" t="str">
-        <f aca="false">IF(E20="","",$B$5+SUM(E$14:F20)-SUM(G$14:H20))</f>
-        <v/>
-      </c>
-      <c r="J20" s="13" t="str">
-        <f aca="false">IF(I20="","",I20/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K20" s="14" t="str">
-        <f aca="false">IF(I20="","",IF(I20&gt;=$B$6,"GOAL HIT",IF(I20&gt;=C20,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
+      <c r="B25" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A25)*($B$7-$B$9)-SUM(B$19:B25)</f>
+        <v>9300</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A25)*($B$8-$B$9)-SUM(B$19:B25)</f>
+        <v>16300</v>
+      </c>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="14" t="str">
+        <f aca="false">IF(E25="","",$B$5+SUM(E$19:F25)-SUM(G$19:H25))</f>
+        <v/>
+      </c>
+      <c r="J25" s="15" t="str">
+        <f aca="false">IF(I25="","",I25/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K25" s="16" t="str">
+        <f aca="false">IF(I25="","",IF(I25&gt;=$B$6,"GOAL HIT",IF(I25&gt;=C25,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12" t="n">
         <v>46356</v>
       </c>
-      <c r="B21" s="11" t="n">
+      <c r="B26" s="13" t="n">
         <v>150</v>
       </c>
-      <c r="C21" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A21)*($B$7-$B$9-$B$10)-SUM(B$14:B21)</f>
-        <v>10050</v>
-      </c>
-      <c r="D21" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A21)*($B$8-$B$9-$B$10)-SUM(B$14:B21)</f>
-        <v>18050</v>
-      </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="12" t="str">
-        <f aca="false">IF(E21="","",$B$5+SUM(E$14:F21)-SUM(G$14:H21))</f>
-        <v/>
-      </c>
-      <c r="J21" s="13" t="str">
-        <f aca="false">IF(I21="","",I21/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K21" s="14" t="str">
-        <f aca="false">IF(I21="","",IF(I21&gt;=$B$6,"GOAL HIT",IF(I21&gt;=C21,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="n">
+      <c r="C26" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A26)*($B$7-$B$9)-SUM(B$19:B26)</f>
+        <v>10150</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A26)*($B$8-$B$9)-SUM(B$19:B26)</f>
+        <v>18150</v>
+      </c>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="14" t="str">
+        <f aca="false">IF(E26="","",$B$5+SUM(E$19:F26)-SUM(G$19:H26))</f>
+        <v/>
+      </c>
+      <c r="J26" s="15" t="str">
+        <f aca="false">IF(I26="","",I26/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K26" s="16" t="str">
+        <f aca="false">IF(I26="","",IF(I26&gt;=$B$6,"GOAL HIT",IF(I26&gt;=C26,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12" t="n">
         <v>46363</v>
       </c>
-      <c r="B22" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A22)*($B$7-$B$9-$B$10)-SUM(B$14:B22)</f>
-        <v>11050</v>
-      </c>
-      <c r="D22" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A22)*($B$8-$B$9-$B$10)-SUM(B$14:B22)</f>
-        <v>20050</v>
-      </c>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="12" t="str">
-        <f aca="false">IF(E22="","",$B$5+SUM(E$14:F22)-SUM(G$14:H22))</f>
-        <v/>
-      </c>
-      <c r="J22" s="13" t="str">
-        <f aca="false">IF(I22="","",I22/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K22" s="14" t="str">
-        <f aca="false">IF(I22="","",IF(I22&gt;=$B$6,"GOAL HIT",IF(I22&gt;=C22,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
+      <c r="B27" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A27)*($B$7-$B$9)-SUM(B$19:B27)</f>
+        <v>11150</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A27)*($B$8-$B$9)-SUM(B$19:B27)</f>
+        <v>20150</v>
+      </c>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="14" t="str">
+        <f aca="false">IF(E27="","",$B$5+SUM(E$19:F27)-SUM(G$19:H27))</f>
+        <v/>
+      </c>
+      <c r="J27" s="15" t="str">
+        <f aca="false">IF(I27="","",I27/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K27" s="16" t="str">
+        <f aca="false">IF(I27="","",IF(I27&gt;=$B$6,"GOAL HIT",IF(I27&gt;=C27,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="n">
         <v>46370</v>
       </c>
-      <c r="B23" s="11" t="n">
+      <c r="B28" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A28)*($B$7-$B$9)-SUM(B$19:B28)</f>
+        <v>12150</v>
+      </c>
+      <c r="D28" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A28)*($B$8-$B$9)-SUM(B$19:B28)</f>
+        <v>22150</v>
+      </c>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="14" t="str">
+        <f aca="false">IF(E28="","",$B$5+SUM(E$19:F28)-SUM(G$19:H28))</f>
+        <v/>
+      </c>
+      <c r="J28" s="15" t="str">
+        <f aca="false">IF(I28="","",I28/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K28" s="16" t="str">
+        <f aca="false">IF(I28="","",IF(I28&gt;=$B$6,"GOAL HIT",IF(I28&gt;=C28,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="n">
+        <v>46377</v>
+      </c>
+      <c r="B29" s="13" t="n">
         <v>300</v>
       </c>
-      <c r="C23" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A23)*($B$7-$B$9-$B$10)-SUM(B$14:B23)</f>
-        <v>11750</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A23)*($B$8-$B$9-$B$10)-SUM(B$14:B23)</f>
-        <v>21750</v>
-      </c>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="12" t="str">
-        <f aca="false">IF(E23="","",$B$5+SUM(E$14:F23)-SUM(G$14:H23))</f>
-        <v/>
-      </c>
-      <c r="J23" s="13" t="str">
-        <f aca="false">IF(I23="","",I23/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K23" s="14" t="str">
-        <f aca="false">IF(I23="","",IF(I23&gt;=$B$6,"GOAL HIT",IF(I23&gt;=C23,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="n">
-        <v>46377</v>
-      </c>
-      <c r="B24" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A24)*($B$7-$B$9-$B$10)-SUM(B$14:B24)</f>
-        <v>12750</v>
-      </c>
-      <c r="D24" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A24)*($B$8-$B$9-$B$10)-SUM(B$14:B24)</f>
-        <v>23750</v>
-      </c>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="12" t="str">
-        <f aca="false">IF(E24="","",$B$5+SUM(E$14:F24)-SUM(G$14:H24))</f>
-        <v/>
-      </c>
-      <c r="J24" s="13" t="str">
-        <f aca="false">IF(I24="","",I24/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K24" s="14" t="str">
-        <f aca="false">IF(I24="","",IF(I24&gt;=$B$6,"GOAL HIT",IF(I24&gt;=C24,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="n">
+      <c r="C29" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A29)*($B$7-$B$9)-SUM(B$19:B29)</f>
+        <v>12850</v>
+      </c>
+      <c r="D29" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A29)*($B$8-$B$9)-SUM(B$19:B29)</f>
+        <v>23850</v>
+      </c>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="14" t="str">
+        <f aca="false">IF(E29="","",$B$5+SUM(E$19:F29)-SUM(G$19:H29))</f>
+        <v/>
+      </c>
+      <c r="J29" s="15" t="str">
+        <f aca="false">IF(I29="","",I29/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K29" s="16" t="str">
+        <f aca="false">IF(I29="","",IF(I29&gt;=$B$6,"GOAL HIT",IF(I29&gt;=C29,"On track","Behind")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12" t="n">
         <v>46384</v>
       </c>
-      <c r="B25" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A25)*($B$7-$B$9-$B$10)-SUM(B$14:B25)</f>
-        <v>13750</v>
-      </c>
-      <c r="D25" s="12" t="n">
-        <f aca="false">$B$5+ROWS(A$14:A25)*($B$8-$B$9-$B$10)-SUM(B$14:B25)</f>
-        <v>25750</v>
-      </c>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="12" t="str">
-        <f aca="false">IF(E25="","",$B$5+SUM(E$14:F25)-SUM(G$14:H25))</f>
-        <v/>
-      </c>
-      <c r="J25" s="13" t="str">
-        <f aca="false">IF(I25="","",I25/$B$6)</f>
-        <v/>
-      </c>
-      <c r="K25" s="14" t="str">
-        <f aca="false">IF(I25="","",IF(I25&gt;=$B$6,"GOAL HIT",IF(I25&gt;=C25,"On track","Behind")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B28" s="15" t="n">
-        <f aca="false">IFERROR(INDEX(A14:A25,MATCH(1,INDEX((C14:C25&gt;=$B$6)*1,0),0)),"Not by Jan 1")</f>
-        <v>46328</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="15" t="n">
-        <f aca="false">IFERROR(INDEX(A14:A25,MATCH(1,INDEX((D14:D25&gt;=$B$6)*1,0),0)),"Not by Jan 1")</f>
-        <v>46314</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="16" t="n">
-        <f aca="false">C25</f>
-        <v>13750</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" s="16" t="n">
-        <f aca="false">D25</f>
-        <v>25750</v>
+      <c r="B30" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A30)*($B$7-$B$9)-SUM(B$19:B30)</f>
+        <v>13850</v>
+      </c>
+      <c r="D30" s="14" t="n">
+        <f aca="false">$B$5+ROWS(A$19:A30)*($B$8-$B$9)-SUM(B$19:B30)</f>
+        <v>25850</v>
+      </c>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
+      <c r="I30" s="14" t="str">
+        <f aca="false">IF(E30="","",$B$5+SUM(E$19:F30)-SUM(G$19:H30))</f>
+        <v/>
+      </c>
+      <c r="J30" s="15" t="str">
+        <f aca="false">IF(I30="","",I30/$B$6)</f>
+        <v/>
+      </c>
+      <c r="K30" s="16" t="str">
+        <f aca="false">IF(I30="","",IF(I30&gt;=$B$6,"GOAL HIT",IF(I30&gt;=C30,"On track","Behind")))</f>
+        <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B32" s="17" t="n">
-        <f aca="false">COUNT(E14:E25)</f>
-        <v>0</v>
+      <c r="A32" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33" s="16" t="str">
-        <f aca="false">IFERROR(AVERAGE(E14:E25),"—")</f>
-        <v>—</v>
+        <v>36</v>
+      </c>
+      <c r="B33" s="17" t="n">
+        <f aca="false">IFERROR(INDEX(A19:A30,MATCH(1,INDEX((C19:C30&gt;=$B$6)*1,0),0)),"Not by Jan 1")</f>
+        <v>46328</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B34" s="16" t="str">
-        <f aca="false">IFERROR(LOOKUP(2,1/(I14:I25&lt;&gt;""),I14:I25),"—")</f>
+        <v>37</v>
+      </c>
+      <c r="B34" s="17" t="n">
+        <f aca="false">IFERROR(INDEX(A19:A30,MATCH(1,INDEX((D19:D30&gt;=$B$6)*1,0),0)),"Not by Jan 1")</f>
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="6" t="n">
+        <f aca="false">C30</f>
+        <v>13850</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" s="6" t="n">
+        <f aca="false">D30</f>
+        <v>25850</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="18" t="n">
+        <f aca="false">COUNT(E19:E30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="6" t="str">
+        <f aca="false">IFERROR(AVERAGE(E19:E30),"—")</f>
         <v>—</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="19" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="19" t="s">
-        <v>37</v>
-      </c>
-    </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="19" t="s">
-        <v>38</v>
+      <c r="A39" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="6" t="str">
+        <f aca="false">IFERROR(LOOKUP(2,1/(I19:I30&lt;&gt;""),I19:I30),"—")</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="20" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K14:K25">
+  <conditionalFormatting sqref="K19:K30">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>"GOAL HIT"</formula>
     </cfRule>
@@ -1623,12 +1739,12 @@
       <formula>"Behind"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C14:D25">
+  <conditionalFormatting sqref="C19:D30">
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>C14&gt;=$B$6</formula>
+      <formula>C19&gt;=$B$6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J14:J25">
+  <conditionalFormatting sqref="J19:J30">
     <cfRule type="dataBar" priority="6">
       <dataBar showValue="1" minLength="10" maxLength="90">
         <cfvo type="num" val="0"/>
@@ -1637,7 +1753,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E873FE8E-40C7-40DA-A231-9BB1D0754C57}</x14:id>
+          <x14:id>{1E11293D-F2B7-44E0-9FCB-50314CF0F030}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -1654,7 +1770,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E873FE8E-40C7-40DA-A231-9BB1D0754C57}">
+          <x14:cfRule type="dataBar" id="{1E11293D-F2B7-44E0-9FCB-50314CF0F030}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -1666,7 +1782,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>J14:J25</xm:sqref>
+          <xm:sqref>J19:J30</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -1693,634 +1809,634 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="B4" s="21" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B5" s="20" t="n">
+        <v>51</v>
+      </c>
+      <c r="B5" s="21" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>43</v>
+      <c r="A6" s="7" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="J8" s="22" t="s">
-        <v>45</v>
+      <c r="B8" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" s="23" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="L9" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="N9" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q9" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="R9" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="S9" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="T9" s="9" t="s">
+      <c r="A9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>55</v>
       </c>
+      <c r="C9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="M9" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="O9" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q9" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="R9" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="S9" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="T9" s="11" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="B10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23" t="n">
+      <c r="A10" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24" t="n">
         <f aca="false">COUNTIF(B10:H10,"x")</f>
         <v>4</v>
       </c>
-      <c r="J10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="K10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="L10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="M10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="N10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="O10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="P10" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q10" s="23" t="n">
+      <c r="J10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="K10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="L10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="M10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="N10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="O10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="P10" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q10" s="24" t="n">
         <f aca="false">COUNTIF(J10:P10,"x")</f>
         <v>7</v>
       </c>
-      <c r="R10" s="23" t="str">
+      <c r="R10" s="24" t="str">
         <f aca="false">IF(I10&gt;=$B$4,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="S10" s="23" t="str">
+      <c r="S10" s="24" t="str">
         <f aca="false">IF(Q10&gt;=$B$5,"Yes","No")</f>
         <v>Yes</v>
       </c>
-      <c r="T10" s="23" t="s">
-        <v>58</v>
+      <c r="T10" s="24" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="n">
+      <c r="A11" s="25" t="n">
         <v>46307</v>
       </c>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="26" t="n">
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+      <c r="I11" s="27" t="n">
         <f aca="false">COUNTIF(B11:H11,"x")</f>
         <v>0</v>
       </c>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
-      <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="26" t="n">
+      <c r="J11" s="26"/>
+      <c r="K11" s="26"/>
+      <c r="L11" s="26"/>
+      <c r="M11" s="26"/>
+      <c r="N11" s="26"/>
+      <c r="O11" s="26"/>
+      <c r="P11" s="26"/>
+      <c r="Q11" s="27" t="n">
         <f aca="false">COUNTIF(J11:P11,"x")</f>
         <v>0</v>
       </c>
-      <c r="R11" s="25" t="str">
+      <c r="R11" s="26" t="str">
         <f aca="false">IF(COUNTA(B11:H11)=0,"",IF(I11&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S11" s="25" t="str">
+      <c r="S11" s="26" t="str">
         <f aca="false">IF(COUNTA(J11:P11)=0,"",IF(Q11&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T11" s="27"/>
+      <c r="T11" s="28"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="n">
+      <c r="A12" s="25" t="n">
         <v>46314</v>
       </c>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="26" t="n">
+      <c r="B12" s="26"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
+      <c r="I12" s="27" t="n">
         <f aca="false">COUNTIF(B12:H12,"x")</f>
         <v>0</v>
       </c>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="25"/>
-      <c r="N12" s="25"/>
-      <c r="O12" s="25"/>
-      <c r="P12" s="25"/>
-      <c r="Q12" s="26" t="n">
+      <c r="J12" s="26"/>
+      <c r="K12" s="26"/>
+      <c r="L12" s="26"/>
+      <c r="M12" s="26"/>
+      <c r="N12" s="26"/>
+      <c r="O12" s="26"/>
+      <c r="P12" s="26"/>
+      <c r="Q12" s="27" t="n">
         <f aca="false">COUNTIF(J12:P12,"x")</f>
         <v>0</v>
       </c>
-      <c r="R12" s="25" t="str">
+      <c r="R12" s="26" t="str">
         <f aca="false">IF(COUNTA(B12:H12)=0,"",IF(I12&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S12" s="25" t="str">
+      <c r="S12" s="26" t="str">
         <f aca="false">IF(COUNTA(J12:P12)=0,"",IF(Q12&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T12" s="27"/>
+      <c r="T12" s="28"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="n">
+      <c r="A13" s="25" t="n">
         <v>46321</v>
       </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="26" t="n">
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="27" t="n">
         <f aca="false">COUNTIF(B13:H13,"x")</f>
         <v>0</v>
       </c>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
-      <c r="O13" s="25"/>
-      <c r="P13" s="25"/>
-      <c r="Q13" s="26" t="n">
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
+      <c r="L13" s="26"/>
+      <c r="M13" s="26"/>
+      <c r="N13" s="26"/>
+      <c r="O13" s="26"/>
+      <c r="P13" s="26"/>
+      <c r="Q13" s="27" t="n">
         <f aca="false">COUNTIF(J13:P13,"x")</f>
         <v>0</v>
       </c>
-      <c r="R13" s="25" t="str">
+      <c r="R13" s="26" t="str">
         <f aca="false">IF(COUNTA(B13:H13)=0,"",IF(I13&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S13" s="25" t="str">
+      <c r="S13" s="26" t="str">
         <f aca="false">IF(COUNTA(J13:P13)=0,"",IF(Q13&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T13" s="27"/>
+      <c r="T13" s="28"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="n">
+      <c r="A14" s="25" t="n">
         <v>46328</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="26" t="n">
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+      <c r="I14" s="27" t="n">
         <f aca="false">COUNTIF(B14:H14,"x")</f>
         <v>0</v>
       </c>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="25"/>
-      <c r="M14" s="25"/>
-      <c r="N14" s="25"/>
-      <c r="O14" s="25"/>
-      <c r="P14" s="25"/>
-      <c r="Q14" s="26" t="n">
+      <c r="J14" s="26"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="26"/>
+      <c r="M14" s="26"/>
+      <c r="N14" s="26"/>
+      <c r="O14" s="26"/>
+      <c r="P14" s="26"/>
+      <c r="Q14" s="27" t="n">
         <f aca="false">COUNTIF(J14:P14,"x")</f>
         <v>0</v>
       </c>
-      <c r="R14" s="25" t="str">
+      <c r="R14" s="26" t="str">
         <f aca="false">IF(COUNTA(B14:H14)=0,"",IF(I14&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S14" s="25" t="str">
+      <c r="S14" s="26" t="str">
         <f aca="false">IF(COUNTA(J14:P14)=0,"",IF(Q14&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T14" s="27"/>
+      <c r="T14" s="28"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="24" t="n">
+      <c r="A15" s="25" t="n">
         <v>46335</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="26" t="n">
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="27" t="n">
         <f aca="false">COUNTIF(B15:H15,"x")</f>
         <v>0</v>
       </c>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="25"/>
-      <c r="N15" s="25"/>
-      <c r="O15" s="25"/>
-      <c r="P15" s="25"/>
-      <c r="Q15" s="26" t="n">
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="26"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="26"/>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="27" t="n">
         <f aca="false">COUNTIF(J15:P15,"x")</f>
         <v>0</v>
       </c>
-      <c r="R15" s="25" t="str">
+      <c r="R15" s="26" t="str">
         <f aca="false">IF(COUNTA(B15:H15)=0,"",IF(I15&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S15" s="25" t="str">
+      <c r="S15" s="26" t="str">
         <f aca="false">IF(COUNTA(J15:P15)=0,"",IF(Q15&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T15" s="27"/>
+      <c r="T15" s="28"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24" t="n">
+      <c r="A16" s="25" t="n">
         <v>46342</v>
       </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="26" t="n">
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="27" t="n">
         <f aca="false">COUNTIF(B16:H16,"x")</f>
         <v>0</v>
       </c>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="25"/>
-      <c r="M16" s="25"/>
-      <c r="N16" s="25"/>
-      <c r="O16" s="25"/>
-      <c r="P16" s="25"/>
-      <c r="Q16" s="26" t="n">
+      <c r="J16" s="26"/>
+      <c r="K16" s="26"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="26"/>
+      <c r="P16" s="26"/>
+      <c r="Q16" s="27" t="n">
         <f aca="false">COUNTIF(J16:P16,"x")</f>
         <v>0</v>
       </c>
-      <c r="R16" s="25" t="str">
+      <c r="R16" s="26" t="str">
         <f aca="false">IF(COUNTA(B16:H16)=0,"",IF(I16&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S16" s="25" t="str">
+      <c r="S16" s="26" t="str">
         <f aca="false">IF(COUNTA(J16:P16)=0,"",IF(Q16&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T16" s="27"/>
+      <c r="T16" s="28"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24" t="n">
+      <c r="A17" s="25" t="n">
         <v>46349</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="26" t="n">
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="27" t="n">
         <f aca="false">COUNTIF(B17:H17,"x")</f>
         <v>0</v>
       </c>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="25"/>
-      <c r="N17" s="25"/>
-      <c r="O17" s="25"/>
-      <c r="P17" s="25"/>
-      <c r="Q17" s="26" t="n">
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
+      <c r="P17" s="26"/>
+      <c r="Q17" s="27" t="n">
         <f aca="false">COUNTIF(J17:P17,"x")</f>
         <v>0</v>
       </c>
-      <c r="R17" s="25" t="str">
+      <c r="R17" s="26" t="str">
         <f aca="false">IF(COUNTA(B17:H17)=0,"",IF(I17&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S17" s="25" t="str">
+      <c r="S17" s="26" t="str">
         <f aca="false">IF(COUNTA(J17:P17)=0,"",IF(Q17&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T17" s="27"/>
+      <c r="T17" s="28"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24" t="n">
+      <c r="A18" s="25" t="n">
         <v>46356</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="26" t="n">
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
+      <c r="I18" s="27" t="n">
         <f aca="false">COUNTIF(B18:H18,"x")</f>
         <v>0</v>
       </c>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="25"/>
-      <c r="M18" s="25"/>
-      <c r="N18" s="25"/>
-      <c r="O18" s="25"/>
-      <c r="P18" s="25"/>
-      <c r="Q18" s="26" t="n">
+      <c r="J18" s="26"/>
+      <c r="K18" s="26"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="26"/>
+      <c r="N18" s="26"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="26"/>
+      <c r="Q18" s="27" t="n">
         <f aca="false">COUNTIF(J18:P18,"x")</f>
         <v>0</v>
       </c>
-      <c r="R18" s="25" t="str">
+      <c r="R18" s="26" t="str">
         <f aca="false">IF(COUNTA(B18:H18)=0,"",IF(I18&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S18" s="25" t="str">
+      <c r="S18" s="26" t="str">
         <f aca="false">IF(COUNTA(J18:P18)=0,"",IF(Q18&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T18" s="27"/>
+      <c r="T18" s="28"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24" t="n">
+      <c r="A19" s="25" t="n">
         <v>46363</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="26" t="n">
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
+      <c r="I19" s="27" t="n">
         <f aca="false">COUNTIF(B19:H19,"x")</f>
         <v>0</v>
       </c>
-      <c r="J19" s="25"/>
-      <c r="K19" s="25"/>
-      <c r="L19" s="25"/>
-      <c r="M19" s="25"/>
-      <c r="N19" s="25"/>
-      <c r="O19" s="25"/>
-      <c r="P19" s="25"/>
-      <c r="Q19" s="26" t="n">
+      <c r="J19" s="26"/>
+      <c r="K19" s="26"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="26"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="26"/>
+      <c r="P19" s="26"/>
+      <c r="Q19" s="27" t="n">
         <f aca="false">COUNTIF(J19:P19,"x")</f>
         <v>0</v>
       </c>
-      <c r="R19" s="25" t="str">
+      <c r="R19" s="26" t="str">
         <f aca="false">IF(COUNTA(B19:H19)=0,"",IF(I19&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S19" s="25" t="str">
+      <c r="S19" s="26" t="str">
         <f aca="false">IF(COUNTA(J19:P19)=0,"",IF(Q19&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T19" s="27"/>
+      <c r="T19" s="28"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="24" t="n">
+      <c r="A20" s="25" t="n">
         <v>46370</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="26" t="n">
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+      <c r="I20" s="27" t="n">
         <f aca="false">COUNTIF(B20:H20,"x")</f>
         <v>0</v>
       </c>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
-      <c r="M20" s="25"/>
-      <c r="N20" s="25"/>
-      <c r="O20" s="25"/>
-      <c r="P20" s="25"/>
-      <c r="Q20" s="26" t="n">
+      <c r="J20" s="26"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="26"/>
+      <c r="O20" s="26"/>
+      <c r="P20" s="26"/>
+      <c r="Q20" s="27" t="n">
         <f aca="false">COUNTIF(J20:P20,"x")</f>
         <v>0</v>
       </c>
-      <c r="R20" s="25" t="str">
+      <c r="R20" s="26" t="str">
         <f aca="false">IF(COUNTA(B20:H20)=0,"",IF(I20&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S20" s="25" t="str">
+      <c r="S20" s="26" t="str">
         <f aca="false">IF(COUNTA(J20:P20)=0,"",IF(Q20&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T20" s="27"/>
+      <c r="T20" s="28"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="24" t="n">
+      <c r="A21" s="25" t="n">
         <v>46377</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="26" t="n">
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="27" t="n">
         <f aca="false">COUNTIF(B21:H21,"x")</f>
         <v>0</v>
       </c>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="25"/>
-      <c r="M21" s="25"/>
-      <c r="N21" s="25"/>
-      <c r="O21" s="25"/>
-      <c r="P21" s="25"/>
-      <c r="Q21" s="26" t="n">
+      <c r="J21" s="26"/>
+      <c r="K21" s="26"/>
+      <c r="L21" s="26"/>
+      <c r="M21" s="26"/>
+      <c r="N21" s="26"/>
+      <c r="O21" s="26"/>
+      <c r="P21" s="26"/>
+      <c r="Q21" s="27" t="n">
         <f aca="false">COUNTIF(J21:P21,"x")</f>
         <v>0</v>
       </c>
-      <c r="R21" s="25" t="str">
+      <c r="R21" s="26" t="str">
         <f aca="false">IF(COUNTA(B21:H21)=0,"",IF(I21&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S21" s="25" t="str">
+      <c r="S21" s="26" t="str">
         <f aca="false">IF(COUNTA(J21:P21)=0,"",IF(Q21&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T21" s="27"/>
+      <c r="T21" s="28"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24" t="n">
+      <c r="A22" s="25" t="n">
         <v>46384</v>
       </c>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="26" t="n">
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="26"/>
+      <c r="I22" s="27" t="n">
         <f aca="false">COUNTIF(B22:H22,"x")</f>
         <v>0</v>
       </c>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
-      <c r="L22" s="25"/>
-      <c r="M22" s="25"/>
-      <c r="N22" s="25"/>
-      <c r="O22" s="25"/>
-      <c r="P22" s="25"/>
-      <c r="Q22" s="26" t="n">
+      <c r="J22" s="26"/>
+      <c r="K22" s="26"/>
+      <c r="L22" s="26"/>
+      <c r="M22" s="26"/>
+      <c r="N22" s="26"/>
+      <c r="O22" s="26"/>
+      <c r="P22" s="26"/>
+      <c r="Q22" s="27" t="n">
         <f aca="false">COUNTIF(J22:P22,"x")</f>
         <v>0</v>
       </c>
-      <c r="R22" s="25" t="str">
+      <c r="R22" s="26" t="str">
         <f aca="false">IF(COUNTA(B22:H22)=0,"",IF(I22&gt;=$B$4,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="S22" s="25" t="str">
+      <c r="S22" s="26" t="str">
         <f aca="false">IF(COUNTA(J22:P22)=0,"",IF(Q22&gt;=$B$5,"Yes","No"))</f>
         <v/>
       </c>
-      <c r="T22" s="27"/>
+      <c r="T22" s="28"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B25" s="28" t="n">
+        <v>69</v>
+      </c>
+      <c r="B25" s="29" t="n">
         <f aca="false">SUM(I11:I22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B26" s="28" t="n">
+        <v>70</v>
+      </c>
+      <c r="B26" s="29" t="n">
         <f aca="false">SUM(Q11:Q22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B27" s="28" t="str">
+        <v>71</v>
+      </c>
+      <c r="B27" s="29" t="str">
         <f aca="false">COUNTIF(R11:R22,"Yes")&amp;" of "&amp;COUNTA(R11:R22)-COUNTBLANK(R11:R22)</f>
         <v>0 of 0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B28" s="28" t="str">
+        <v>72</v>
+      </c>
+      <c r="B28" s="29" t="str">
         <f aca="false">COUNTIF(S11:S22,"Yes")&amp;" of "&amp;COUNTA(S11:S22)-COUNTBLANK(S11:S22)</f>
         <v>0 of 0</v>
       </c>

</xml_diff>